<commit_message>
Append 24-08-2026 SNGP purchase to JS_Zindigi_SNGP_Trading_Analysis.xlsx
One new Trade Data row (1 share @ 102.61, commission 0.21, matching the
real contract note) following the exact formula pattern of every existing
row; Summary sheet's SUM ranges extended from row 32 to row 33 accordingly.
LibreOffice recalculation could not complete in this sandbox (a pre-existing
environment limitation -- the original file already ships with no cached
formula values either, confirmed against git history, so this doesn't
introduce a new inconsistency); any real Excel/Sheets session recalculates
on open as usual.
</commit_message>
<xml_diff>
--- a/JS_Zindigi_SNGP_Trading_Analysis.xlsx
+++ b/JS_Zindigi_SNGP_Trading_Analysis.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fee Settings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Trade Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fee Settings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S32"/>
+  <dimension ref="A1:S33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2782,6 +2782,78 @@
       </c>
       <c r="S32" s="2" t="n"/>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>24-Aug-2026</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>SNGP</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>SNGPL</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>102.61</v>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="H33" s="2">
+        <f>D33*E33</f>
+        <v/>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="2">
+        <f>H33+F33+I33</f>
+        <v/>
+      </c>
+      <c r="K33" s="2">
+        <f>D33*G33</f>
+        <v/>
+      </c>
+      <c r="L33" s="2">
+        <f>D33*G33*0.002</f>
+        <v/>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="2">
+        <f>K33-L33-M33</f>
+        <v/>
+      </c>
+      <c r="O33" s="2">
+        <f>N33-J33</f>
+        <v/>
+      </c>
+      <c r="P33" s="2">
+        <f>MAX(O33,0)*0.15</f>
+        <v/>
+      </c>
+      <c r="Q33" s="2">
+        <f>O33-P33</f>
+        <v/>
+      </c>
+      <c r="R33" s="2">
+        <f>(J33+L33+M33)/D33</f>
+        <v/>
+      </c>
+      <c r="S33" s="2" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2968,7 +3040,7 @@
         </is>
       </c>
       <c r="B2" s="2">
-        <f>SUM('Trade Data'!D2:D32)</f>
+        <f>SUM('Trade Data'!D2:D33)</f>
         <v/>
       </c>
     </row>
@@ -2979,7 +3051,7 @@
         </is>
       </c>
       <c r="B3" s="2">
-        <f>SUM('Trade Data'!H2:H32)</f>
+        <f>SUM('Trade Data'!H2:H33)</f>
         <v/>
       </c>
     </row>
@@ -2990,7 +3062,7 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <f>SUM('Trade Data'!F2:F32)</f>
+        <f>SUM('Trade Data'!F2:F33)</f>
         <v/>
       </c>
     </row>
@@ -3001,7 +3073,7 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <f>SUM('Trade Data'!J2:J32)</f>
+        <f>SUM('Trade Data'!J2:J33)</f>
         <v/>
       </c>
     </row>
@@ -3012,7 +3084,7 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <f>SUM('Trade Data'!K2:K32)</f>
+        <f>SUM('Trade Data'!K2:K33)</f>
         <v/>
       </c>
     </row>
@@ -3023,7 +3095,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <f>SUM('Trade Data'!L2:L32)</f>
+        <f>SUM('Trade Data'!L2:L33)</f>
         <v/>
       </c>
     </row>
@@ -3034,7 +3106,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <f>SUM('Trade Data'!N2:N32)</f>
+        <f>SUM('Trade Data'!N2:N33)</f>
         <v/>
       </c>
     </row>
@@ -3045,7 +3117,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <f>SUM('Trade Data'!O2:O32)</f>
+        <f>SUM('Trade Data'!O2:O33)</f>
         <v/>
       </c>
     </row>
@@ -3056,7 +3128,7 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <f>SUM('Trade Data'!P2:P32)</f>
+        <f>SUM('Trade Data'!P2:P33)</f>
         <v/>
       </c>
     </row>
@@ -3067,7 +3139,7 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <f>SUM('Trade Data'!Q2:Q32)</f>
+        <f>SUM('Trade Data'!Q2:Q33)</f>
         <v/>
       </c>
     </row>
@@ -3110,7 +3182,7 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <f>SUM('Trade Data'!J2:J32)/B2+SUM('Trade Data'!L2:L32)/B2</f>
+        <f>SUM('Trade Data'!J2:J33)/B2+SUM('Trade Data'!L2:L33)/B2</f>
         <v/>
       </c>
     </row>

</xml_diff>